<commit_message>
fix(excel-suite-pel): correggi nome funzione test_calendario_03 (test_evento_con_invitati)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/suite_test_pel.xlsx
+++ b/suite_test_pel.xlsx
@@ -1205,7 +1205,7 @@
       </c>
       <c r="D7" s="31" t="inlineStr">
         <is>
-          <t>test_creazione_invio_evento</t>
+          <t>test_evento_con_invitati</t>
         </is>
       </c>
       <c r="E7" s="32" t="inlineStr">
@@ -2169,7 +2169,7 @@
       <c r="B5" s="58" t="inlineStr">
         <is>
           <t>test_calendario_03.py
-test_creazione_invio_evento</t>
+test_evento_con_invitati</t>
         </is>
       </c>
       <c r="C5" s="59" t="inlineStr">

</xml_diff>

<commit_message>
refactor(pel): rinumera test calendario 01-10, aggiorna Excel suite
- test_calendario_05: era test_08 (giornata intera)
- test_calendario_06: era test_09 (promemoria)
- test_calendario_07: era test_15 (disponibilità occupato)
- test_calendario_08: era test_16 (disponibilità libero)
- test_calendario_09: era test_17 (pianificazione invitato occupato)
- test_calendario_10: era test_18 (pianificazione multi-invitati)
- Aggiornati riferimenti interni (screenshot, print) alla nuova numerazione
- genera_excel_suite_pel.py: aggiornata lista test con nuova numerazione
- Rigenera suite_test_pel.xlsx: 14 test totali (2 Login + 10 Calendario + 2 Impostazioni)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/suite_test_pel.xlsx
+++ b/suite_test_pel.xlsx
@@ -906,11 +906,11 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Test sul modulo Calendario PEL: creazione/modifica eventi, ricorrenze, viste, navigazione, giornata intera, promemoria, ricerca, luogo, rich text, calendario assegnato e disponibilità.</t>
+          <t>Test sul modulo Calendario PEL: creazione/modifica eventi, ricorrenze, invitati, import/export ICS, giornata intera, promemoria, disponibilità occupato/libero e vista pianificazione multi-invitati.</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="C8" s="13" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D8" s="14" t="n"/>
     </row>
@@ -959,7 +959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1273,7 +1273,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="154" customHeight="1">
+    <row r="9" ht="126" customHeight="1">
       <c r="A9" s="29" t="n">
         <v>7</v>
       </c>
@@ -1289,147 +1289,15 @@
       </c>
       <c r="D9" s="31" t="inlineStr">
         <is>
-          <t>test_crea_calendario_personalizzato</t>
+          <t>test_evento_giornata_intera</t>
         </is>
       </c>
       <c r="E9" s="32" t="inlineStr">
         <is>
-          <t>Verifica la creazione di un nuovo calendario con nome e colore, poi lo elimina.</t>
+          <t>Verifica la creazione di un evento con toggle 'Giornata intera' attivato.</t>
         </is>
       </c>
       <c r="F9" s="33" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Aprire 'Gestione calendario'.
-4. Cliccare 'Nuovo' per creare un nuovo calendario.
-5. Inserire un nome univoco (con timestamp).
-6. Selezionare un colore tra quelli disponibili.
-7. Salvare il calendario.
-8. Verificare il toast di conferma.
-9. Verificare che il calendario sia visibile nella sidebar.
-10. Scattare screenshot.
-11. Eliminare il calendario (click destro → Elimina calendario, cleanup).</t>
-        </is>
-      </c>
-      <c r="G9" s="34" t="inlineStr">
-        <is>
-          <t>Il nuovo calendario è creato e appare nella sidebar. Il toast di conferma è visibile. Il calendario viene eliminato correttamente nel cleanup.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="140" customHeight="1">
-      <c r="A10" s="35" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="35" t="inlineStr">
-        <is>
-          <t>Calendario</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>test_calendario_06.py</t>
-        </is>
-      </c>
-      <c r="D10" s="25" t="inlineStr">
-        <is>
-          <t>test_cambio_vista_calendario</t>
-        </is>
-      </c>
-      <c r="E10" s="26" t="inlineStr">
-        <is>
-          <t>Verifica il cambio tra le diverse viste del calendario: Giorno, Mese, Eventi, Settimana.</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Cliccare il pulsante vista 'Giorno' ([title='Giorno']).
-4. Scattare screenshot della vista Giorno.
-5. Cliccare il pulsante vista 'Mese' ([title='Mese']).
-6. Scattare screenshot della vista Mese.
-7. Cliccare il pulsante vista 'Eventi' ([title='Eventi']).
-8. Scattare screenshot della vista Eventi.
-9. Cliccare il pulsante vista 'Settimana' ([title='Settimana']).
-10. Scattare screenshot finale.</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="inlineStr">
-        <is>
-          <t>Il calendario cambia correttamente tra le viste Giorno, Mese, Eventi e Settimana senza errori. Per ogni cambio lo screenshot mostra il layout corretto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="126" customHeight="1">
-      <c r="A11" s="29" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>Calendario</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr">
-        <is>
-          <t>test_calendario_07.py</t>
-        </is>
-      </c>
-      <c r="D11" s="31" t="inlineStr">
-        <is>
-          <t>test_navigazione_periodi_calendario</t>
-        </is>
-      </c>
-      <c r="E11" s="32" t="inlineStr">
-        <is>
-          <t>Verifica la navigazione del calendario tramite mini-calendar e pulsante 'Oggi'.</t>
-        </is>
-      </c>
-      <c r="F11" s="33" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Leggere il primo giorno della settimana corrente (.fc-col-header-cell).
-4. Cliccare 'Next' nella mini-calendar per avanzare di un mese.
-5. Cliccare il primo giorno disponibile del mese successivo.
-6. Verificare che la main view si sia aggiornata (primo giorno diverso).
-7. Cliccare il pulsante 'Oggi'.
-8. Scattare screenshot.
-9. Verificare il ritorno alla settimana corrente (primo giorno uguale all'iniziale, assert).</t>
-        </is>
-      </c>
-      <c r="G11" s="34" t="inlineStr">
-        <is>
-          <t>La navigazione tramite mini-calendar aggiorna la main view. Il pulsante 'Oggi' riporta correttamente alla settimana corrente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="126" customHeight="1">
-      <c r="A12" s="35" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" s="35" t="inlineStr">
-        <is>
-          <t>Calendario</t>
-        </is>
-      </c>
-      <c r="C12" s="24" t="inlineStr">
-        <is>
-          <t>test_calendario_08.py</t>
-        </is>
-      </c>
-      <c r="D12" s="25" t="inlineStr">
-        <is>
-          <t>test_evento_giornata_intera</t>
-        </is>
-      </c>
-      <c r="E12" s="26" t="inlineStr">
-        <is>
-          <t>Verifica la creazione di un evento con toggle 'Giornata intera' attivato.</t>
-        </is>
-      </c>
-      <c r="F12" s="27" t="inlineStr">
         <is>
           <t>1. Accedere con credenziali valide.
 2. Navigare nella sezione Calendario.
@@ -1442,303 +1310,83 @@
 9. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
-      <c r="G12" s="28" t="inlineStr">
+      <c r="G9" s="34" t="inlineStr">
         <is>
           <t>L'evento è creato come evento 'Giornata intera' ed è visibile nel calendario (nella banda all-day o nella griglia). Il cleanup elimina l'evento correttamente.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="154" customHeight="1">
-      <c r="A13" s="29" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" s="29" t="inlineStr">
+    <row r="10" ht="168" customHeight="1">
+      <c r="A10" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>Calendario</t>
         </is>
       </c>
-      <c r="C13" s="30" t="inlineStr">
-        <is>
-          <t>test_calendario_09.py</t>
-        </is>
-      </c>
-      <c r="D13" s="31" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>test_calendario_06.py</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
         <is>
           <t>test_evento_con_promemoria</t>
         </is>
       </c>
-      <c r="E13" s="32" t="inlineStr">
+      <c r="E10" s="26" t="inlineStr">
         <is>
           <t>Verifica la configurazione e il salvataggio di un promemoria per un evento del calendario.</t>
         </is>
       </c>
-      <c r="F13" s="33" t="inlineStr">
+      <c r="F10" s="27" t="inlineStr">
         <is>
           <t>1. Accedere con credenziali valide.
 2. Navigare nella sezione Calendario.
 3. Cliccare 'Nuovo evento'.
 4. Inserire un titolo univoco.
-5. Cliccare 'Aggiungi promemoria'.
-6. Configurare il tipo di notifica (email) e inserire l'indirizzo.
-7. Salvare il dialog promemoria.
-8. Salvare l'evento.
-9. Verificare che l'evento sia visibile nel calendario (.fc-event).
-10. Scattare screenshot.
-11. Eliminare l'evento (cleanup).</t>
-        </is>
-      </c>
-      <c r="G13" s="34" t="inlineStr">
-        <is>
-          <t>Il promemoria è configurato e l'evento è salvato correttamente. L'evento è visibile nella griglia del calendario. Il cleanup elimina l'evento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="140" customHeight="1">
-      <c r="A14" s="35" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" s="35" t="inlineStr">
-        <is>
-          <t>Calendario</t>
-        </is>
-      </c>
-      <c r="C14" s="24" t="inlineStr">
-        <is>
-          <t>test_calendario_10.py</t>
-        </is>
-      </c>
-      <c r="D14" s="25" t="inlineStr">
-        <is>
-          <t>test_ricerca_nel_calendario</t>
-        </is>
-      </c>
-      <c r="E14" s="26" t="inlineStr">
-        <is>
-          <t>Verifica la funzione di ricerca eventi nel calendario tramite la barra di ricerca.</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Creare un evento con titolo univoco (timestamp).
-4. Salvare l'evento.
-5. Cercare l'evento tramite la barra 'Cerca nel calendario'.
-6. Premere Enter per avviare la ricerca.
-7. Verificare che il testo univoco sia trovato.
-8. Fallback: se la ricerca restituisce spinner, verificare tramite vista Eventi.
-9. Scattare screenshot.
-10. Eliminare l'evento (cleanup).</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="inlineStr">
-        <is>
-          <t>L'evento con il titolo univoco è trovato tramite ricerca o visibile nella vista Eventi. Il cleanup elimina l'evento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="126" customHeight="1">
-      <c r="A15" s="29" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" s="29" t="inlineStr">
-        <is>
-          <t>Calendario</t>
-        </is>
-      </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>test_calendario_11.py</t>
-        </is>
-      </c>
-      <c r="D15" s="31" t="inlineStr">
-        <is>
-          <t>test_evento_luogo_indirizzo</t>
-        </is>
-      </c>
-      <c r="E15" s="32" t="inlineStr">
-        <is>
-          <t>Verifica la creazione di un evento con tipo luogo 'Indirizzo' e il salvataggio del campo location.</t>
-        </is>
-      </c>
-      <c r="F15" s="33" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Cliccare 'Nuovo evento'.
-4. Inserire un titolo univoco.
-5. Inserire un indirizzo fisico nel campo luogo (es. 'Via Roma 1, Milano').
-6. Salvare l'evento.
-7. Aprire l'evento dalla griglia e verificare che l'indirizzo sia presente nel popup.
-8. Scattare screenshot.
-9. Eliminare l'evento (cleanup).</t>
-        </is>
-      </c>
-      <c r="G15" s="34" t="inlineStr">
-        <is>
-          <t>Il luogo 'Via Roma 1, Milano' è salvato correttamente e visibile nel popup dell'evento. Il cleanup elimina l'evento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="126" customHeight="1">
-      <c r="A16" s="35" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" s="35" t="inlineStr">
-        <is>
-          <t>Calendario</t>
-        </is>
-      </c>
-      <c r="C16" s="24" t="inlineStr">
-        <is>
-          <t>test_calendario_12.py</t>
-        </is>
-      </c>
-      <c r="D16" s="25" t="inlineStr">
-        <is>
-          <t>test_evento_luogo_link</t>
-        </is>
-      </c>
-      <c r="E16" s="26" t="inlineStr">
-        <is>
-          <t>Verifica la creazione di un evento con URL meeting come luogo e il salvataggio del campo.</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Cliccare 'Nuovo evento'.
-4. Inserire un titolo univoco.
-5. Inserire un URL meeting nel campo luogo (es. 'https://meet.example.com/test-room').
-6. Salvare l'evento.
-7. Aprire l'evento dalla griglia e verificare che l'URL sia presente nel popup.
-8. Scattare screenshot.
-9. Eliminare l'evento (cleanup).</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="inlineStr">
-        <is>
-          <t>L'URL meeting è salvato correttamente e visibile (parzialmente o intero) nel popup dell'evento. Il cleanup elimina l'evento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="168" customHeight="1">
-      <c r="A17" s="29" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" s="29" t="inlineStr">
-        <is>
-          <t>Calendario</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="inlineStr">
-        <is>
-          <t>test_calendario_13.py</t>
-        </is>
-      </c>
-      <c r="D17" s="31" t="inlineStr">
-        <is>
-          <t>test_evento_corpo_rich_text</t>
-        </is>
-      </c>
-      <c r="E17" s="32" t="inlineStr">
-        <is>
-          <t>Verifica la creazione di un evento con corpo in rich text (grassetto + lista) tramite suneditor.</t>
-        </is>
-      </c>
-      <c r="F17" s="33" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Cliccare 'Nuovo evento'.
-4. Inserire un titolo univoco.
-5. Espandere a fullscreen per accedere al rich text editor.
-6. Cliccare nell'area editable del suneditor.
-7. Attivare il grassetto (toolbar o Ctrl+B) e digitare il testo.
-8. Aggiungere una voce di lista.
+5. Chiudere banner cookie se presente.
+6. Cliccare 'Aggiungi promemoria'.
+7. Configurare il tipo di notifica (email) e inserire l'indirizzo.
+8. Salvare il dialog promemoria.
 9. Salvare l'evento.
-10. Aprire l'evento e verificare che il testo in grassetto sia visibile nel popup.
+10. Verificare che l'evento sia visibile nel calendario (.fc-event).
 11. Scattare screenshot.
 12. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
-      <c r="G17" s="34" t="inlineStr">
-        <is>
-          <t>Il testo in grassetto inserito tramite rich text editor è salvato e visibile nel popup evento. Il cleanup elimina l'evento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="154" customHeight="1">
-      <c r="A18" s="35" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" s="35" t="inlineStr">
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>Il promemoria è configurato e l'evento è salvato correttamente. L'evento è visibile nella griglia del calendario. Il cleanup elimina l'evento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="168" customHeight="1">
+      <c r="A11" s="29" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
         <is>
           <t>Calendario</t>
         </is>
       </c>
-      <c r="C18" s="24" t="inlineStr">
-        <is>
-          <t>test_calendario_14.py</t>
-        </is>
-      </c>
-      <c r="D18" s="25" t="inlineStr">
-        <is>
-          <t>test_assegna_calendario_specifico</t>
-        </is>
-      </c>
-      <c r="E18" s="26" t="inlineStr">
-        <is>
-          <t>Verifica la creazione di un evento assegnandolo a un calendario specifico.</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Cliccare 'Nuovo evento'.
-4. Inserire un titolo univoco.
-5. Espandere a fullscreen per accedere al campo 'Calendario assegnato'.
-6. Aprire il combobox del calendario (default 'Personale').
-7. Selezionare un'opzione diversa dall'attuale se disponibile.
-8. Salvare l'evento.
-9. Verificare che l'evento sia visibile nel calendario.
-10. Scattare screenshot.
-11. Eliminare l'evento (cleanup).</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="inlineStr">
-        <is>
-          <t>L'evento è creato e assegnato al calendario selezionato. L'evento è visibile nella griglia del calendario. Il cleanup elimina l'evento correttamente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="168" customHeight="1">
-      <c r="A19" s="29" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" s="29" t="inlineStr">
-        <is>
-          <t>Calendario</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr">
-        <is>
-          <t>test_calendario_15.py</t>
-        </is>
-      </c>
-      <c r="D19" s="31" t="inlineStr">
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>test_calendario_07.py</t>
+        </is>
+      </c>
+      <c r="D11" s="31" t="inlineStr">
         <is>
           <t>test_disponibilita_occupato</t>
         </is>
       </c>
-      <c r="E19" s="32" t="inlineStr">
+      <c r="E11" s="32" t="inlineStr">
         <is>
           <t>Verifica che un evento con 'Mostrati come occupato' ON salvi correttamente la preferenza.</t>
         </is>
       </c>
-      <c r="F19" s="33" t="inlineStr">
+      <c r="F11" s="33" t="inlineStr">
         <is>
           <t>1. Accedere con credenziali valide.
 2. Navigare nella sezione Calendario.
@@ -1754,79 +1402,164 @@
 12. Eliminare l'evento nel finally (cleanup).</t>
         </is>
       </c>
-      <c r="G19" s="34" t="inlineStr">
+      <c r="G11" s="34" t="inlineStr">
         <is>
           <t>Il toggle 'Mostrati come occupato' è checked (ON) alla riapertura dell'evento, confermando che la preferenza è stata salvata correttamente.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="112" customHeight="1">
-      <c r="A20" s="35" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" s="35" t="inlineStr">
+    <row r="12" ht="98" customHeight="1">
+      <c r="A12" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>Calendario</t>
         </is>
       </c>
-      <c r="C20" s="24" t="inlineStr">
-        <is>
-          <t>test_calendario_16.py</t>
-        </is>
-      </c>
-      <c r="D20" s="25" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>test_calendario_08.py</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="inlineStr">
         <is>
           <t>test_disponibilita_libero</t>
         </is>
       </c>
-      <c r="E20" s="26" t="inlineStr">
+      <c r="E12" s="26" t="inlineStr">
         <is>
           <t>Verifica che un evento con 'Mostrati come occupato' OFF non renda lo slot occupato nella vista pianificazione.</t>
         </is>
       </c>
-      <c r="F20" s="27" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Creare evento A con 'Mostrati come occupato' OFF (Libero) alle 14:00-15:00.
+      <c r="F12" s="27" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare evento A con 'Mostrati come occupato' OFF (Libero) con orario futuro.
 3. Creare evento B alla stessa ora aggiungendo se stesso come invitato.
 4. Aprire la vista di pianificazione disponibilità (aru-button.planning-button).
-5. Verificare che lo slot 14:00-15:00 NON risulti 'Occupato' (exact=True).
+5. Verificare che lo slot NON risulti 'Occupato' (exact=True).
 6. Scattare screenshot.
-7. Chiudere la vista pianificazione e annullare l'evento B.
-8. Eliminare entrambi gli eventi nel finally (cleanup).</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="inlineStr">
-        <is>
-          <t>Lo slot 14:00-15:00 non risulta 'Occupato' nella vista pianificazione, confermando che l'evento con 'Mostrati come occupato' OFF non impatta la disponibilità.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="168" customHeight="1">
-      <c r="A21" s="36" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" s="36" t="inlineStr">
+7. Nel finally: chiudere dialog aperti, eliminare entrambi gli eventi (cleanup).</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>Lo slot non risulta 'Occupato' nella vista pianificazione, confermando che l'evento con 'Mostrati come occupato' OFF non impatta la disponibilità.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="112" customHeight="1">
+      <c r="A13" s="29" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>Calendario</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>test_calendario_09.py</t>
+        </is>
+      </c>
+      <c r="D13" s="31" t="inlineStr">
+        <is>
+          <t>test_pianificazione_invitato_occupato</t>
+        </is>
+      </c>
+      <c r="E13" s="32" t="inlineStr">
+        <is>
+          <t>Verifica che nella vista pianificazione disponibilità uno slot risulti occupato quando l'invitato ha un evento con 'Mostrati come occupato' ON.</t>
+        </is>
+      </c>
+      <c r="F13" s="33" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare evento A con orario futuro (+2h) — 'Mostrati come occupato' ON (default).
+3. Aprire un nuovo evento B alla stessa ora, aggiungere se stesso come invitato.
+4. Aprire la vista pianificazione disponibilità (aru-button.planning-button).
+5. Identificare la modale 'Disponibilità degli invitati' (pane con 'Tu (').
+6. Verificare la presenza di un blocco colorato (rosa/rosso) nella griglia.
+7. Scattare screenshot.
+8. Nel finally: chiudere dialog aperti, eliminare evento A e annullare evento B (cleanup).</t>
+        </is>
+      </c>
+      <c r="G13" s="34" t="inlineStr">
+        <is>
+          <t>La modale pianificazione mostra un blocco colorato nella riga dell'invitato, confermando che l'evento A con 'Mostrati come occupato' ON occupa lo slot. Il cleanup elimina correttamente entrambi gli eventi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="140" customHeight="1">
+      <c r="A14" s="35" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>Calendario</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>test_calendario_10.py</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>test_pianificazione_multi_invitati</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>Verifica la vista pianificazione disponibilità con più invitati, confermando che tutti appaiono nella griglia.</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare nella sezione Calendario.
+3. Creare un nuovo evento con titolo univoco.
+4. Aggiungere destinatario_principale come invitato 1.
+5. Aggiungere destinatario_secondario come invitato 2.
+6. Aprire la vista pianificazione (link 'Pianifica e mostra disponibilità invitati' o aru-button.planning-button).
+7. Verificare che invitato 1 sia visibile nella griglia pianificazione.
+8. Verificare che invitato 2 sia visibile nella griglia pianificazione.
+9. Scattare screenshot.
+10. Nel finally: chiudere dialog aperti, eliminare l'evento (cleanup).</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>La vista pianificazione mostra entrambi gli invitati nella griglia. Il cleanup chiude il dialog e rimuove l'evento correttamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="168" customHeight="1">
+      <c r="A15" s="36" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="36" t="inlineStr">
         <is>
           <t>Impostazioni</t>
         </is>
       </c>
-      <c r="C21" s="37" t="inlineStr">
+      <c r="C15" s="37" t="inlineStr">
         <is>
           <t>test_impostazioni_calendari.py</t>
         </is>
       </c>
-      <c r="D21" s="38" t="inlineStr">
+      <c r="D15" s="38" t="inlineStr">
         <is>
           <t>test_impostazioni_luogo_predefinito</t>
         </is>
       </c>
-      <c r="E21" s="39" t="inlineStr">
+      <c r="E15" s="39" t="inlineStr">
         <is>
           <t>S1: Imposta un luogo predefinito nelle impostazioni calendario e verifica che venga pre-compilato alla creazione di un nuovo evento.</t>
         </is>
       </c>
-      <c r="F21" s="40" t="inlineStr">
+      <c r="F15" s="40" t="inlineStr">
         <is>
           <t>1. Accedere con credenziali valide.
 2. Navigare a /settings/calendars/customization tramite URL diretto.
@@ -1842,37 +1575,37 @@
 12. Ripristinare il luogo vuoto nelle impostazioni (cleanup).</t>
         </is>
       </c>
-      <c r="G21" s="41" t="inlineStr">
+      <c r="G15" s="41" t="inlineStr">
         <is>
           <t>La pagina impostazioni calendario è accessibile. Se il campo luogo è presente, il valore viene salvato e letto nel form del nuovo evento. L'impostazione viene ripristinata al termine.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="140" customHeight="1">
-      <c r="A22" s="42" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="42" t="inlineStr">
+    <row r="16" ht="140" customHeight="1">
+      <c r="A16" s="42" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
         <is>
           <t>Impostazioni</t>
         </is>
       </c>
-      <c r="C22" s="24" t="inlineStr">
+      <c r="C16" s="24" t="inlineStr">
         <is>
           <t>test_impostazioni_calendari.py</t>
         </is>
       </c>
-      <c r="D22" s="25" t="inlineStr">
+      <c r="D16" s="25" t="inlineStr">
         <is>
           <t>test_impostazioni_visualizzazione_predefinita</t>
         </is>
       </c>
-      <c r="E22" s="26" t="inlineStr">
+      <c r="E16" s="26" t="inlineStr">
         <is>
           <t>S2: Cambia la visualizzazione predefinita del calendario e verifica che il calendario si apra con quella vista.</t>
         </is>
       </c>
-      <c r="F22" s="27" t="inlineStr">
+      <c r="F16" s="27" t="inlineStr">
         <is>
           <t>1. Accedere con credenziali valide.
 2. Navigare a /settings/calendars/customization tramite URL diretto.
@@ -1886,7 +1619,7 @@
 10. Ripristinare la visualizzazione predefinita originale (cleanup).</t>
         </is>
       </c>
-      <c r="G22" s="28" t="inlineStr">
+      <c r="G16" s="28" t="inlineStr">
         <is>
           <t>Se la selezione della vista 'Mese' è riuscita: il calendario si apre in vista Mese. Se il combobox usa shadow DOM non interagibile: la pagina impostazioni è accessibile (PASS con fallback).</t>
         </is>
@@ -2037,7 +1770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2051,7 +1784,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="55" t="inlineStr">
         <is>
-          <t>MODULO: CALENDARIO  –  16 Casi di Test</t>
+          <t>MODULO: CALENDARIO  –  10 Casi di Test</t>
         </is>
       </c>
     </row>
@@ -2230,130 +1963,22 @@
       </c>
       <c r="F6" s="54" t="inlineStr"/>
     </row>
-    <row r="7" ht="154" customHeight="1">
+    <row r="7" ht="126" customHeight="1">
       <c r="A7" s="57" t="n">
         <v>7</v>
       </c>
       <c r="B7" s="58" t="inlineStr">
         <is>
           <t>test_calendario_05.py
-test_crea_calendario_personalizzato</t>
+test_evento_giornata_intera</t>
         </is>
       </c>
       <c r="C7" s="59" t="inlineStr">
         <is>
-          <t>Verifica la creazione di un nuovo calendario con nome e colore, poi lo elimina.</t>
+          <t>Verifica la creazione di un evento con toggle 'Giornata intera' attivato.</t>
         </is>
       </c>
       <c r="D7" s="60" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Aprire 'Gestione calendario'.
-4. Cliccare 'Nuovo' per creare un nuovo calendario.
-5. Inserire un nome univoco (con timestamp).
-6. Selezionare un colore tra quelli disponibili.
-7. Salvare il calendario.
-8. Verificare il toast di conferma.
-9. Verificare che il calendario sia visibile nella sidebar.
-10. Scattare screenshot.
-11. Eliminare il calendario (click destro → Elimina calendario, cleanup).</t>
-        </is>
-      </c>
-      <c r="E7" s="34" t="inlineStr">
-        <is>
-          <t>Il nuovo calendario è creato e appare nella sidebar. Il toast di conferma è visibile. Il calendario viene eliminato correttamente nel cleanup.</t>
-        </is>
-      </c>
-      <c r="F7" s="61" t="inlineStr"/>
-    </row>
-    <row r="8" ht="140" customHeight="1">
-      <c r="A8" s="62" t="n">
-        <v>8</v>
-      </c>
-      <c r="B8" s="51" t="inlineStr">
-        <is>
-          <t>test_calendario_06.py
-test_cambio_vista_calendario</t>
-        </is>
-      </c>
-      <c r="C8" s="52" t="inlineStr">
-        <is>
-          <t>Verifica il cambio tra le diverse viste del calendario: Giorno, Mese, Eventi, Settimana.</t>
-        </is>
-      </c>
-      <c r="D8" s="53" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Cliccare il pulsante vista 'Giorno' ([title='Giorno']).
-4. Scattare screenshot della vista Giorno.
-5. Cliccare il pulsante vista 'Mese' ([title='Mese']).
-6. Scattare screenshot della vista Mese.
-7. Cliccare il pulsante vista 'Eventi' ([title='Eventi']).
-8. Scattare screenshot della vista Eventi.
-9. Cliccare il pulsante vista 'Settimana' ([title='Settimana']).
-10. Scattare screenshot finale.</t>
-        </is>
-      </c>
-      <c r="E8" s="28" t="inlineStr">
-        <is>
-          <t>Il calendario cambia correttamente tra le viste Giorno, Mese, Eventi e Settimana senza errori. Per ogni cambio lo screenshot mostra il layout corretto.</t>
-        </is>
-      </c>
-      <c r="F8" s="54" t="inlineStr"/>
-    </row>
-    <row r="9" ht="126" customHeight="1">
-      <c r="A9" s="57" t="n">
-        <v>9</v>
-      </c>
-      <c r="B9" s="58" t="inlineStr">
-        <is>
-          <t>test_calendario_07.py
-test_navigazione_periodi_calendario</t>
-        </is>
-      </c>
-      <c r="C9" s="59" t="inlineStr">
-        <is>
-          <t>Verifica la navigazione del calendario tramite mini-calendar e pulsante 'Oggi'.</t>
-        </is>
-      </c>
-      <c r="D9" s="60" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Leggere il primo giorno della settimana corrente (.fc-col-header-cell).
-4. Cliccare 'Next' nella mini-calendar per avanzare di un mese.
-5. Cliccare il primo giorno disponibile del mese successivo.
-6. Verificare che la main view si sia aggiornata (primo giorno diverso).
-7. Cliccare il pulsante 'Oggi'.
-8. Scattare screenshot.
-9. Verificare il ritorno alla settimana corrente (primo giorno uguale all'iniziale, assert).</t>
-        </is>
-      </c>
-      <c r="E9" s="34" t="inlineStr">
-        <is>
-          <t>La navigazione tramite mini-calendar aggiorna la main view. Il pulsante 'Oggi' riporta correttamente alla settimana corrente.</t>
-        </is>
-      </c>
-      <c r="F9" s="61" t="inlineStr"/>
-    </row>
-    <row r="10" ht="126" customHeight="1">
-      <c r="A10" s="62" t="n">
-        <v>10</v>
-      </c>
-      <c r="B10" s="51" t="inlineStr">
-        <is>
-          <t>test_calendario_08.py
-test_evento_giornata_intera</t>
-        </is>
-      </c>
-      <c r="C10" s="52" t="inlineStr">
-        <is>
-          <t>Verifica la creazione di un evento con toggle 'Giornata intera' attivato.</t>
-        </is>
-      </c>
-      <c r="D10" s="53" t="inlineStr">
         <is>
           <t>1. Accedere con credenziali valide.
 2. Navigare nella sezione Calendario.
@@ -2366,247 +1991,67 @@
 9. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
-      <c r="E10" s="28" t="inlineStr">
+      <c r="E7" s="34" t="inlineStr">
         <is>
           <t>L'evento è creato come evento 'Giornata intera' ed è visibile nel calendario (nella banda all-day o nella griglia). Il cleanup elimina l'evento correttamente.</t>
         </is>
       </c>
-      <c r="F10" s="54" t="inlineStr"/>
-    </row>
-    <row r="11" ht="154" customHeight="1">
-      <c r="A11" s="57" t="n">
-        <v>11</v>
-      </c>
-      <c r="B11" s="58" t="inlineStr">
-        <is>
-          <t>test_calendario_09.py
+      <c r="F7" s="61" t="inlineStr"/>
+    </row>
+    <row r="8" ht="168" customHeight="1">
+      <c r="A8" s="62" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" s="51" t="inlineStr">
+        <is>
+          <t>test_calendario_06.py
 test_evento_con_promemoria</t>
         </is>
       </c>
-      <c r="C11" s="59" t="inlineStr">
+      <c r="C8" s="52" t="inlineStr">
         <is>
           <t>Verifica la configurazione e il salvataggio di un promemoria per un evento del calendario.</t>
         </is>
       </c>
-      <c r="D11" s="60" t="inlineStr">
+      <c r="D8" s="53" t="inlineStr">
         <is>
           <t>1. Accedere con credenziali valide.
 2. Navigare nella sezione Calendario.
 3. Cliccare 'Nuovo evento'.
 4. Inserire un titolo univoco.
-5. Cliccare 'Aggiungi promemoria'.
-6. Configurare il tipo di notifica (email) e inserire l'indirizzo.
-7. Salvare il dialog promemoria.
-8. Salvare l'evento.
-9. Verificare che l'evento sia visibile nel calendario (.fc-event).
-10. Scattare screenshot.
-11. Eliminare l'evento (cleanup).</t>
-        </is>
-      </c>
-      <c r="E11" s="34" t="inlineStr">
-        <is>
-          <t>Il promemoria è configurato e l'evento è salvato correttamente. L'evento è visibile nella griglia del calendario. Il cleanup elimina l'evento.</t>
-        </is>
-      </c>
-      <c r="F11" s="61" t="inlineStr"/>
-    </row>
-    <row r="12" ht="140" customHeight="1">
-      <c r="A12" s="62" t="n">
-        <v>12</v>
-      </c>
-      <c r="B12" s="51" t="inlineStr">
-        <is>
-          <t>test_calendario_10.py
-test_ricerca_nel_calendario</t>
-        </is>
-      </c>
-      <c r="C12" s="52" t="inlineStr">
-        <is>
-          <t>Verifica la funzione di ricerca eventi nel calendario tramite la barra di ricerca.</t>
-        </is>
-      </c>
-      <c r="D12" s="53" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Creare un evento con titolo univoco (timestamp).
-4. Salvare l'evento.
-5. Cercare l'evento tramite la barra 'Cerca nel calendario'.
-6. Premere Enter per avviare la ricerca.
-7. Verificare che il testo univoco sia trovato.
-8. Fallback: se la ricerca restituisce spinner, verificare tramite vista Eventi.
-9. Scattare screenshot.
-10. Eliminare l'evento (cleanup).</t>
-        </is>
-      </c>
-      <c r="E12" s="28" t="inlineStr">
-        <is>
-          <t>L'evento con il titolo univoco è trovato tramite ricerca o visibile nella vista Eventi. Il cleanup elimina l'evento.</t>
-        </is>
-      </c>
-      <c r="F12" s="54" t="inlineStr"/>
-    </row>
-    <row r="13" ht="126" customHeight="1">
-      <c r="A13" s="57" t="n">
-        <v>13</v>
-      </c>
-      <c r="B13" s="58" t="inlineStr">
-        <is>
-          <t>test_calendario_11.py
-test_evento_luogo_indirizzo</t>
-        </is>
-      </c>
-      <c r="C13" s="59" t="inlineStr">
-        <is>
-          <t>Verifica la creazione di un evento con tipo luogo 'Indirizzo' e il salvataggio del campo location.</t>
-        </is>
-      </c>
-      <c r="D13" s="60" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Cliccare 'Nuovo evento'.
-4. Inserire un titolo univoco.
-5. Inserire un indirizzo fisico nel campo luogo (es. 'Via Roma 1, Milano').
-6. Salvare l'evento.
-7. Aprire l'evento dalla griglia e verificare che l'indirizzo sia presente nel popup.
-8. Scattare screenshot.
-9. Eliminare l'evento (cleanup).</t>
-        </is>
-      </c>
-      <c r="E13" s="34" t="inlineStr">
-        <is>
-          <t>Il luogo 'Via Roma 1, Milano' è salvato correttamente e visibile nel popup dell'evento. Il cleanup elimina l'evento.</t>
-        </is>
-      </c>
-      <c r="F13" s="61" t="inlineStr"/>
-    </row>
-    <row r="14" ht="126" customHeight="1">
-      <c r="A14" s="62" t="n">
-        <v>14</v>
-      </c>
-      <c r="B14" s="51" t="inlineStr">
-        <is>
-          <t>test_calendario_12.py
-test_evento_luogo_link</t>
-        </is>
-      </c>
-      <c r="C14" s="52" t="inlineStr">
-        <is>
-          <t>Verifica la creazione di un evento con URL meeting come luogo e il salvataggio del campo.</t>
-        </is>
-      </c>
-      <c r="D14" s="53" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Cliccare 'Nuovo evento'.
-4. Inserire un titolo univoco.
-5. Inserire un URL meeting nel campo luogo (es. 'https://meet.example.com/test-room').
-6. Salvare l'evento.
-7. Aprire l'evento dalla griglia e verificare che l'URL sia presente nel popup.
-8. Scattare screenshot.
-9. Eliminare l'evento (cleanup).</t>
-        </is>
-      </c>
-      <c r="E14" s="28" t="inlineStr">
-        <is>
-          <t>L'URL meeting è salvato correttamente e visibile (parzialmente o intero) nel popup dell'evento. Il cleanup elimina l'evento.</t>
-        </is>
-      </c>
-      <c r="F14" s="54" t="inlineStr"/>
-    </row>
-    <row r="15" ht="168" customHeight="1">
-      <c r="A15" s="57" t="n">
-        <v>15</v>
-      </c>
-      <c r="B15" s="58" t="inlineStr">
-        <is>
-          <t>test_calendario_13.py
-test_evento_corpo_rich_text</t>
-        </is>
-      </c>
-      <c r="C15" s="59" t="inlineStr">
-        <is>
-          <t>Verifica la creazione di un evento con corpo in rich text (grassetto + lista) tramite suneditor.</t>
-        </is>
-      </c>
-      <c r="D15" s="60" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Cliccare 'Nuovo evento'.
-4. Inserire un titolo univoco.
-5. Espandere a fullscreen per accedere al rich text editor.
-6. Cliccare nell'area editable del suneditor.
-7. Attivare il grassetto (toolbar o Ctrl+B) e digitare il testo.
-8. Aggiungere una voce di lista.
+5. Chiudere banner cookie se presente.
+6. Cliccare 'Aggiungi promemoria'.
+7. Configurare il tipo di notifica (email) e inserire l'indirizzo.
+8. Salvare il dialog promemoria.
 9. Salvare l'evento.
-10. Aprire l'evento e verificare che il testo in grassetto sia visibile nel popup.
+10. Verificare che l'evento sia visibile nel calendario (.fc-event).
 11. Scattare screenshot.
 12. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
-      <c r="E15" s="34" t="inlineStr">
-        <is>
-          <t>Il testo in grassetto inserito tramite rich text editor è salvato e visibile nel popup evento. Il cleanup elimina l'evento.</t>
-        </is>
-      </c>
-      <c r="F15" s="61" t="inlineStr"/>
-    </row>
-    <row r="16" ht="154" customHeight="1">
-      <c r="A16" s="62" t="n">
-        <v>16</v>
-      </c>
-      <c r="B16" s="51" t="inlineStr">
-        <is>
-          <t>test_calendario_14.py
-test_assegna_calendario_specifico</t>
-        </is>
-      </c>
-      <c r="C16" s="52" t="inlineStr">
-        <is>
-          <t>Verifica la creazione di un evento assegnandolo a un calendario specifico.</t>
-        </is>
-      </c>
-      <c r="D16" s="53" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Navigare nella sezione Calendario.
-3. Cliccare 'Nuovo evento'.
-4. Inserire un titolo univoco.
-5. Espandere a fullscreen per accedere al campo 'Calendario assegnato'.
-6. Aprire il combobox del calendario (default 'Personale').
-7. Selezionare un'opzione diversa dall'attuale se disponibile.
-8. Salvare l'evento.
-9. Verificare che l'evento sia visibile nel calendario.
-10. Scattare screenshot.
-11. Eliminare l'evento (cleanup).</t>
-        </is>
-      </c>
-      <c r="E16" s="28" t="inlineStr">
-        <is>
-          <t>L'evento è creato e assegnato al calendario selezionato. L'evento è visibile nella griglia del calendario. Il cleanup elimina l'evento correttamente.</t>
-        </is>
-      </c>
-      <c r="F16" s="54" t="inlineStr"/>
-    </row>
-    <row r="17" ht="168" customHeight="1">
-      <c r="A17" s="57" t="n">
-        <v>17</v>
-      </c>
-      <c r="B17" s="58" t="inlineStr">
-        <is>
-          <t>test_calendario_15.py
+      <c r="E8" s="28" t="inlineStr">
+        <is>
+          <t>Il promemoria è configurato e l'evento è salvato correttamente. L'evento è visibile nella griglia del calendario. Il cleanup elimina l'evento.</t>
+        </is>
+      </c>
+      <c r="F8" s="54" t="inlineStr"/>
+    </row>
+    <row r="9" ht="168" customHeight="1">
+      <c r="A9" s="57" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" s="58" t="inlineStr">
+        <is>
+          <t>test_calendario_07.py
 test_disponibilita_occupato</t>
         </is>
       </c>
-      <c r="C17" s="59" t="inlineStr">
+      <c r="C9" s="59" t="inlineStr">
         <is>
           <t>Verifica che un evento con 'Mostrati come occupato' ON salvi correttamente la preferenza.</t>
         </is>
       </c>
-      <c r="D17" s="60" t="inlineStr">
+      <c r="D9" s="60" t="inlineStr">
         <is>
           <t>1. Accedere con credenziali valide.
 2. Navigare nella sezione Calendario.
@@ -2622,46 +2067,115 @@
 12. Eliminare l'evento nel finally (cleanup).</t>
         </is>
       </c>
-      <c r="E17" s="34" t="inlineStr">
+      <c r="E9" s="34" t="inlineStr">
         <is>
           <t>Il toggle 'Mostrati come occupato' è checked (ON) alla riapertura dell'evento, confermando che la preferenza è stata salvata correttamente.</t>
         </is>
       </c>
-      <c r="F17" s="61" t="inlineStr"/>
-    </row>
-    <row r="18" ht="112" customHeight="1">
-      <c r="A18" s="62" t="n">
-        <v>18</v>
-      </c>
-      <c r="B18" s="51" t="inlineStr">
-        <is>
-          <t>test_calendario_16.py
+      <c r="F9" s="61" t="inlineStr"/>
+    </row>
+    <row r="10" ht="98" customHeight="1">
+      <c r="A10" s="62" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" s="51" t="inlineStr">
+        <is>
+          <t>test_calendario_08.py
 test_disponibilita_libero</t>
         </is>
       </c>
-      <c r="C18" s="52" t="inlineStr">
+      <c r="C10" s="52" t="inlineStr">
         <is>
           <t>Verifica che un evento con 'Mostrati come occupato' OFF non renda lo slot occupato nella vista pianificazione.</t>
         </is>
       </c>
-      <c r="D18" s="53" t="inlineStr">
-        <is>
-          <t>1. Accedere con credenziali valide.
-2. Creare evento A con 'Mostrati come occupato' OFF (Libero) alle 14:00-15:00.
+      <c r="D10" s="53" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare evento A con 'Mostrati come occupato' OFF (Libero) con orario futuro.
 3. Creare evento B alla stessa ora aggiungendo se stesso come invitato.
 4. Aprire la vista di pianificazione disponibilità (aru-button.planning-button).
-5. Verificare che lo slot 14:00-15:00 NON risulti 'Occupato' (exact=True).
+5. Verificare che lo slot NON risulti 'Occupato' (exact=True).
 6. Scattare screenshot.
-7. Chiudere la vista pianificazione e annullare l'evento B.
-8. Eliminare entrambi gli eventi nel finally (cleanup).</t>
-        </is>
-      </c>
-      <c r="E18" s="28" t="inlineStr">
-        <is>
-          <t>Lo slot 14:00-15:00 non risulta 'Occupato' nella vista pianificazione, confermando che l'evento con 'Mostrati come occupato' OFF non impatta la disponibilità.</t>
-        </is>
-      </c>
-      <c r="F18" s="54" t="inlineStr"/>
+7. Nel finally: chiudere dialog aperti, eliminare entrambi gli eventi (cleanup).</t>
+        </is>
+      </c>
+      <c r="E10" s="28" t="inlineStr">
+        <is>
+          <t>Lo slot non risulta 'Occupato' nella vista pianificazione, confermando che l'evento con 'Mostrati come occupato' OFF non impatta la disponibilità.</t>
+        </is>
+      </c>
+      <c r="F10" s="54" t="inlineStr"/>
+    </row>
+    <row r="11" ht="112" customHeight="1">
+      <c r="A11" s="57" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" s="58" t="inlineStr">
+        <is>
+          <t>test_calendario_09.py
+test_pianificazione_invitato_occupato</t>
+        </is>
+      </c>
+      <c r="C11" s="59" t="inlineStr">
+        <is>
+          <t>Verifica che nella vista pianificazione disponibilità uno slot risulti occupato quando l'invitato ha un evento con 'Mostrati come occupato' ON.</t>
+        </is>
+      </c>
+      <c r="D11" s="60" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare evento A con orario futuro (+2h) — 'Mostrati come occupato' ON (default).
+3. Aprire un nuovo evento B alla stessa ora, aggiungere se stesso come invitato.
+4. Aprire la vista pianificazione disponibilità (aru-button.planning-button).
+5. Identificare la modale 'Disponibilità degli invitati' (pane con 'Tu (').
+6. Verificare la presenza di un blocco colorato (rosa/rosso) nella griglia.
+7. Scattare screenshot.
+8. Nel finally: chiudere dialog aperti, eliminare evento A e annullare evento B (cleanup).</t>
+        </is>
+      </c>
+      <c r="E11" s="34" t="inlineStr">
+        <is>
+          <t>La modale pianificazione mostra un blocco colorato nella riga dell'invitato, confermando che l'evento A con 'Mostrati come occupato' ON occupa lo slot. Il cleanup elimina correttamente entrambi gli eventi.</t>
+        </is>
+      </c>
+      <c r="F11" s="61" t="inlineStr"/>
+    </row>
+    <row r="12" ht="140" customHeight="1">
+      <c r="A12" s="62" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" s="51" t="inlineStr">
+        <is>
+          <t>test_calendario_10.py
+test_pianificazione_multi_invitati</t>
+        </is>
+      </c>
+      <c r="C12" s="52" t="inlineStr">
+        <is>
+          <t>Verifica la vista pianificazione disponibilità con più invitati, confermando che tutti appaiono nella griglia.</t>
+        </is>
+      </c>
+      <c r="D12" s="53" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare nella sezione Calendario.
+3. Creare un nuovo evento con titolo univoco.
+4. Aggiungere destinatario_principale come invitato 1.
+5. Aggiungere destinatario_secondario come invitato 2.
+6. Aprire la vista pianificazione (link 'Pianifica e mostra disponibilità invitati' o aru-button.planning-button).
+7. Verificare che invitato 1 sia visibile nella griglia pianificazione.
+8. Verificare che invitato 2 sia visibile nella griglia pianificazione.
+9. Scattare screenshot.
+10. Nel finally: chiudere dialog aperti, eliminare l'evento (cleanup).</t>
+        </is>
+      </c>
+      <c r="E12" s="28" t="inlineStr">
+        <is>
+          <t>La vista pianificazione mostra entrambi gli invitati nella griglia. Il cleanup chiude il dialog e rimuove l'evento correttamente.</t>
+        </is>
+      </c>
+      <c r="F12" s="54" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2729,7 +2243,7 @@
     </row>
     <row r="3" ht="168" customHeight="1">
       <c r="A3" s="65" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B3" s="66" t="inlineStr">
         <is>
@@ -2767,7 +2281,7 @@
     </row>
     <row r="4" ht="140" customHeight="1">
       <c r="A4" s="70" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B4" s="51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(readme): documenta il testbook Excel e come rigenerarlo
Il README non menzionava da nessuna parte gli script
genera_excel_suite*.py ne' i file .xlsx che producono, nonostante
siano il testbook di riferimento per la QA manuale. Aggiunta una
sezione dedicata con lo scopo di ciascun generatore e il comando per
rigenerarlo, oltre ai riferimenti nella struttura del progetto.

Rigenerati suite_test_pec_mobile.xlsx e suite_test_pel.xlsx per
verificare che i comandi documentati funzionino davvero.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/suite_test_pel.xlsx
+++ b/suite_test_pel.xlsx
@@ -906,11 +906,11 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Test sul modulo Calendario PEL: creazione/modifica eventi, ricorrenze, invitati, import/export ICS, giornata intera, promemoria, disponibilità occupato/libero e vista pianificazione multi-invitati.</t>
+          <t>Test sul modulo Calendario PEL: creazione/modifica eventi, ricorrenze, invitati, import/export ICS, giornata intera, promemoria, disponibilità, pianificazione multi-invitati, conflitto sala riunioni, gestione invitati e drag-and-drop.</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="C8" s="13" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D8" s="14" t="n"/>
     </row>
@@ -959,7 +959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1535,31 +1535,160 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="168" customHeight="1">
-      <c r="A15" s="36" t="n">
+    <row r="15" ht="112" customHeight="1">
+      <c r="A15" s="29" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="36" t="inlineStr">
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>Calendario</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>test_calendario_11.py</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
+        <is>
+          <t>test_conflitto_sala_riunioni</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>Verifica che la sala riunioni risulti non selezionabile quando è già prenotata nello stesso orario.</t>
+        </is>
+      </c>
+      <c r="F15" s="33" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare Evento A con sala riunioni disponibile (orario futuro +3h).
+3. Leggere il nome della sala auto-selezionata per Evento A.
+4. Salvare Evento A.
+5. Creare Evento B allo stesso orario e selezionare il tipo 'Sala riunioni'.
+6. Verificare che la sala sia read-only, disabilitata o assente (conflitto rilevato).
+7. Scattare screenshot.
+8. Nel finally: chiudere form aperti, eliminare Evento A ed Evento B (cleanup).</t>
+        </is>
+      </c>
+      <c r="G15" s="34" t="inlineStr">
+        <is>
+          <t>Il sistema rileva il conflitto: la sala prenotata in Evento A risulta non selezionabile (read-only, disabled o non proposta) in Evento B allo stesso orario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="126" customHeight="1">
+      <c r="A16" s="35" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>Calendario</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>test_calendario_12.py</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="inlineStr">
+        <is>
+          <t>test_invitati_aggiungi_rimuovi</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>Verifica che sia possibile aggiungere due invitati a un evento e successivamente rimuoverne uno.</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un evento con invitato_1 e invitato_2 → Invia.
+3. Riaprire l'evento dal calendario → form di modifica fullscreen.
+4. Verificare che entrambi gli invitati siano presenti nella lista.
+5. Rimuovere invitato_1 tramite il pulsante × (hover + click, più strategie).
+6. Verificare nella lista invitati che invitato_1 sia assente e invitato_2 ancora presente.
+7. Salvare e gestire il dialogo 'Vuoi informare gli invitati?' → Non inviare.
+8. Scattare screenshot.
+9. Nel finally: chiudere form aperti, eliminare l'evento (cleanup).</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="inlineStr">
+        <is>
+          <t>Dopo la rimozione, la lista invitati nel form contiene solo invitato_2. Il salvataggio avviene senza errori. Il cleanup elimina l'evento correttamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="140" customHeight="1">
+      <c r="A17" s="29" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>Calendario</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>test_calendario_13.py</t>
+        </is>
+      </c>
+      <c r="D17" s="31" t="inlineStr">
+        <is>
+          <t>test_sposta_evento_drag</t>
+        </is>
+      </c>
+      <c r="E17" s="32" t="inlineStr">
+        <is>
+          <t>Verifica che un evento possa essere spostato su un altro giorno tramite drag-and-drop nella vista Settimana.</t>
+        </is>
+      </c>
+      <c r="F17" s="33" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare alla vista Settimana del calendario.
+3. Creare un evento semplice (nessun invitato) alle 10:00-11:00 oggi.
+4. Calcolare il giorno target (±2 giorni, nella stessa settimana visualizzata).
+5. Trovare l'evento nella griglia (.fc-event).
+6. Eseguire il drag lento (25 passi, 30 ms/passo) verso la colonna del giorno target.
+7. Attendere che FullCalendar aggiorni la posizione dell'evento.
+8. Verificare tramite bounding box che il centro X dell'evento ricada nella colonna target.
+9. Scattare screenshot pre/post drag.
+10. Nel finally: chiudere overlay aperti, eliminare l'evento (cleanup).</t>
+        </is>
+      </c>
+      <c r="G17" s="34" t="inlineStr">
+        <is>
+          <t>Dopo il drag, il centro X dell'evento è compreso nei limiti della colonna del giorno target. Il test PASSED conferma che FullCalendar ha registrato lo spostamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="168" customHeight="1">
+      <c r="A18" s="36" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="36" t="inlineStr">
         <is>
           <t>Impostazioni</t>
         </is>
       </c>
-      <c r="C15" s="37" t="inlineStr">
+      <c r="C18" s="37" t="inlineStr">
         <is>
           <t>test_impostazioni_calendari.py</t>
         </is>
       </c>
-      <c r="D15" s="38" t="inlineStr">
+      <c r="D18" s="38" t="inlineStr">
         <is>
           <t>test_impostazioni_luogo_predefinito</t>
         </is>
       </c>
-      <c r="E15" s="39" t="inlineStr">
+      <c r="E18" s="39" t="inlineStr">
         <is>
           <t>S1: Imposta un luogo predefinito nelle impostazioni calendario e verifica che venga pre-compilato alla creazione di un nuovo evento.</t>
         </is>
       </c>
-      <c r="F15" s="40" t="inlineStr">
+      <c r="F18" s="40" t="inlineStr">
         <is>
           <t>1. Accedere con credenziali valide.
 2. Navigare a /settings/calendars/customization tramite URL diretto.
@@ -1575,37 +1704,37 @@
 12. Ripristinare il luogo vuoto nelle impostazioni (cleanup).</t>
         </is>
       </c>
-      <c r="G15" s="41" t="inlineStr">
+      <c r="G18" s="41" t="inlineStr">
         <is>
           <t>La pagina impostazioni calendario è accessibile. Se il campo luogo è presente, il valore viene salvato e letto nel form del nuovo evento. L'impostazione viene ripristinata al termine.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="140" customHeight="1">
-      <c r="A16" s="42" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" s="42" t="inlineStr">
+    <row r="19" ht="140" customHeight="1">
+      <c r="A19" s="42" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t>Impostazioni</t>
         </is>
       </c>
-      <c r="C16" s="24" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>test_impostazioni_calendari.py</t>
         </is>
       </c>
-      <c r="D16" s="25" t="inlineStr">
+      <c r="D19" s="25" t="inlineStr">
         <is>
           <t>test_impostazioni_visualizzazione_predefinita</t>
         </is>
       </c>
-      <c r="E16" s="26" t="inlineStr">
+      <c r="E19" s="26" t="inlineStr">
         <is>
           <t>S2: Cambia la visualizzazione predefinita del calendario e verifica che il calendario si apra con quella vista.</t>
         </is>
       </c>
-      <c r="F16" s="27" t="inlineStr">
+      <c r="F19" s="27" t="inlineStr">
         <is>
           <t>1. Accedere con credenziali valide.
 2. Navigare a /settings/calendars/customization tramite URL diretto.
@@ -1619,7 +1748,7 @@
 10. Ripristinare la visualizzazione predefinita originale (cleanup).</t>
         </is>
       </c>
-      <c r="G16" s="28" t="inlineStr">
+      <c r="G19" s="28" t="inlineStr">
         <is>
           <t>Se la selezione della vista 'Mese' è riuscita: il calendario si apre in vista Mese. Se il combobox usa shadow DOM non interagibile: la pagina impostazioni è accessibile (PASS con fallback).</t>
         </is>
@@ -1770,7 +1899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1784,7 +1913,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="55" t="inlineStr">
         <is>
-          <t>MODULO: CALENDARIO  –  10 Casi di Test</t>
+          <t>MODULO: CALENDARIO  –  13 Casi di Test</t>
         </is>
       </c>
     </row>
@@ -2176,6 +2305,111 @@
         </is>
       </c>
       <c r="F12" s="54" t="inlineStr"/>
+    </row>
+    <row r="13" ht="112" customHeight="1">
+      <c r="A13" s="57" t="n">
+        <v>13</v>
+      </c>
+      <c r="B13" s="58" t="inlineStr">
+        <is>
+          <t>test_calendario_11.py
+test_conflitto_sala_riunioni</t>
+        </is>
+      </c>
+      <c r="C13" s="59" t="inlineStr">
+        <is>
+          <t>Verifica che la sala riunioni risulti non selezionabile quando è già prenotata nello stesso orario.</t>
+        </is>
+      </c>
+      <c r="D13" s="60" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare Evento A con sala riunioni disponibile (orario futuro +3h).
+3. Leggere il nome della sala auto-selezionata per Evento A.
+4. Salvare Evento A.
+5. Creare Evento B allo stesso orario e selezionare il tipo 'Sala riunioni'.
+6. Verificare che la sala sia read-only, disabilitata o assente (conflitto rilevato).
+7. Scattare screenshot.
+8. Nel finally: chiudere form aperti, eliminare Evento A ed Evento B (cleanup).</t>
+        </is>
+      </c>
+      <c r="E13" s="34" t="inlineStr">
+        <is>
+          <t>Il sistema rileva il conflitto: la sala prenotata in Evento A risulta non selezionabile (read-only, disabled o non proposta) in Evento B allo stesso orario.</t>
+        </is>
+      </c>
+      <c r="F13" s="61" t="inlineStr"/>
+    </row>
+    <row r="14" ht="126" customHeight="1">
+      <c r="A14" s="62" t="n">
+        <v>14</v>
+      </c>
+      <c r="B14" s="51" t="inlineStr">
+        <is>
+          <t>test_calendario_12.py
+test_invitati_aggiungi_rimuovi</t>
+        </is>
+      </c>
+      <c r="C14" s="52" t="inlineStr">
+        <is>
+          <t>Verifica che sia possibile aggiungere due invitati a un evento e successivamente rimuoverne uno.</t>
+        </is>
+      </c>
+      <c r="D14" s="53" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un evento con invitato_1 e invitato_2 → Invia.
+3. Riaprire l'evento dal calendario → form di modifica fullscreen.
+4. Verificare che entrambi gli invitati siano presenti nella lista.
+5. Rimuovere invitato_1 tramite il pulsante × (hover + click, più strategie).
+6. Verificare nella lista invitati che invitato_1 sia assente e invitato_2 ancora presente.
+7. Salvare e gestire il dialogo 'Vuoi informare gli invitati?' → Non inviare.
+8. Scattare screenshot.
+9. Nel finally: chiudere form aperti, eliminare l'evento (cleanup).</t>
+        </is>
+      </c>
+      <c r="E14" s="28" t="inlineStr">
+        <is>
+          <t>Dopo la rimozione, la lista invitati nel form contiene solo invitato_2. Il salvataggio avviene senza errori. Il cleanup elimina l'evento correttamente.</t>
+        </is>
+      </c>
+      <c r="F14" s="54" t="inlineStr"/>
+    </row>
+    <row r="15" ht="140" customHeight="1">
+      <c r="A15" s="57" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" s="58" t="inlineStr">
+        <is>
+          <t>test_calendario_13.py
+test_sposta_evento_drag</t>
+        </is>
+      </c>
+      <c r="C15" s="59" t="inlineStr">
+        <is>
+          <t>Verifica che un evento possa essere spostato su un altro giorno tramite drag-and-drop nella vista Settimana.</t>
+        </is>
+      </c>
+      <c r="D15" s="60" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare alla vista Settimana del calendario.
+3. Creare un evento semplice (nessun invitato) alle 10:00-11:00 oggi.
+4. Calcolare il giorno target (±2 giorni, nella stessa settimana visualizzata).
+5. Trovare l'evento nella griglia (.fc-event).
+6. Eseguire il drag lento (25 passi, 30 ms/passo) verso la colonna del giorno target.
+7. Attendere che FullCalendar aggiorni la posizione dell'evento.
+8. Verificare tramite bounding box che il centro X dell'evento ricada nella colonna target.
+9. Scattare screenshot pre/post drag.
+10. Nel finally: chiudere overlay aperti, eliminare l'evento (cleanup).</t>
+        </is>
+      </c>
+      <c r="E15" s="34" t="inlineStr">
+        <is>
+          <t>Dopo il drag, il centro X dell'evento è compreso nei limiti della colonna del giorno target. Il test PASSED conferma che FullCalendar ha registrato lo spostamento.</t>
+        </is>
+      </c>
+      <c r="F15" s="61" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2243,7 +2477,7 @@
     </row>
     <row r="3" ht="168" customHeight="1">
       <c r="A3" s="65" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B3" s="66" t="inlineStr">
         <is>
@@ -2281,7 +2515,7 @@
     </row>
     <row r="4" ht="140" customHeight="1">
       <c r="A4" s="70" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B4" s="51" t="inlineStr">
         <is>

</xml_diff>